<commit_message>
Add token link to chat sheet token rows
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013vbY3qGkzmvkM4RiAXuEBt
</commit_message>
<xml_diff>
--- a/FlexiGenie_Webinar_Chat_Sheet.xlsx
+++ b/FlexiGenie_Webinar_Chat_Sheet.xlsx
@@ -3426,7 +3426,7 @@
       </c>
       <c r="C153" s="6" t="inlineStr">
         <is>
-          <t>Share your contact number as well for the token link</t>
+          <t>Token Link: https://sb.flexifunnels.com/reserve2k – Share your contact number as well</t>
         </is>
       </c>
       <c r="D153" s="13" t="inlineStr">
@@ -5340,7 +5340,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>{Name}, you can reserve your seat with a token payment. Type 1 / share your contact number and our team will send you the token link.</t>
+          <t>{Name}, you can reserve your seat with a token payment here: https://sb.flexifunnels.com/reserve2k. Share your contact number and our team will help you with the remaining payment.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Use English-only lines in chat sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013vbY3qGkzmvkM4RiAXuEBt
</commit_message>
<xml_diff>
--- a/FlexiGenie_Webinar_Chat_Sheet.xlsx
+++ b/FlexiGenie_Webinar_Chat_Sheet.xlsx
@@ -578,7 +578,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Hi everyone 👋 Welcome! Kahan se join kar rahe ho? Drop your city 👇</t>
+          <t>Hi everyone 👋 Welcome! Where are you joining from? Drop your city 👇</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>600+ log live hain abhi 🔥</t>
+          <t>600+ people live right now 🔥</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -616,8 +616,8 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Type 1 – Business hai, online le jaana hai
-Type 2 – Side income chahiye
+          <t>Type 1 – I have a business and want to take it online
+Type 2 – I want a side income
 Type 3 – Just exploring</t>
         </is>
       </c>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Confidence aaya? Can you do this yourself now? Type Yes</t>
+          <t>Feeling confident? Can you do this yourself now? Type Yes</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Questions note karte jao 📝 Sir will answer at the end. Keep your WhatsApp number ready too 😉</t>
+          <t>Keep noting down your questions 📝 Sir will answer them at the end. Keep your WhatsApp number ready too 😉</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>EMI chahiye? Drop your number – our team will find the easiest EMI plan for you in 2 minutes ✅</t>
+          <t>Need EMI? Drop your number – our team will find the easiest EMI plan for you in 2 minutes ✅</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Sochte sochte seat chali jaayegi 😅 Drop your number – our team will call you right now</t>
+          <t>Don't lose your seat while you're still thinking 😅 Drop your number – our team will call you right now</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Job ke saath kaise karein? Drop your number – our team will plan your 1 hour/day routine with you ⏰</t>
+          <t>Wondering how to do this alongside your job? Drop your number – our team will plan your 1 hour/day routine with you ⏰</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>Deal pakki? 🤝 Seal it – drop your number</t>
+          <t>Is it a deal? 🤝 Seal it – drop your number</t>
         </is>
       </c>
       <c r="D111" s="11" t="inlineStr">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="C124" s="11" t="inlineStr">
         <is>
-          <t>Last call. Aaj number nahi diya, toh kal bhi yahi sochoge. Drop it now 👇</t>
+          <t>Last call. If you don't drop your number today, you'll still be thinking about it tomorrow. Drop it now 👇</t>
         </is>
       </c>
       <c r="D124" s="11" t="inlineStr">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>EMI chahiye? Drop your number – our team will find the easiest EMI plan for you in 2 minutes ✅</t>
+          <t>Need EMI? Drop your number – our team will find the easiest EMI plan for you in 2 minutes ✅</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Job ke saath kaise karein? Drop your number – our team will plan your 1 hour/day routine with you ⏰</t>
+          <t>Wondering how to do this alongside your job? Drop your number – our team will plan your 1 hour/day routine with you ⏰</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Deal pakki? 🤝 Seal it – drop your number</t>
+          <t>Is it a deal? 🤝 Seal it – drop your number</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -3449,7 +3449,7 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Sochte sochte seat chali jaayegi 😅 Drop your number – our team will call you right now</t>
+          <t>Don't lose your seat while you're still thinking 😅 Drop your number – our team will call you right now</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Last call. Aaj number nahi diya, toh kal bhi yahi sochoge. Drop it now 👇</t>
+          <t>Last call. If you don't drop your number today, you'll still be thinking about it tomorrow. Drop it now 👇</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Remove emojis from chat sheet lines
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013vbY3qGkzmvkM4RiAXuEBt
</commit_message>
<xml_diff>
--- a/FlexiGenie_Webinar_Chat_Sheet.xlsx
+++ b/FlexiGenie_Webinar_Chat_Sheet.xlsx
@@ -578,7 +578,7 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Hi everyone 👋 Welcome! Where are you joining from? Drop your city 👇</t>
+          <t>Hi everyone, welcome! Where are you joining from? Drop your city in the chat</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>600+ people live right now 🔥</t>
+          <t>600+ people live right now</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Launch your entire online business in 10 minutes – just by chatting from your phone 📱</t>
+          <t>Launch your entire online business in 10 minutes – just by chatting from your phone</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
@@ -656,7 +656,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Sounds unbelievable? Type 1 if you're being honest 😄</t>
+          <t>Sounds unbelievable? Type 1 if you're being honest</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>2 days FREE access already sent on your email ✅ Type Yes if you got it</t>
+          <t>2 days FREE access already sent on your email. Type Yes if you got it</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -713,7 +713,7 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Stay till the end 👉 FREE 1-on-1 consultation + special announcement 🎁</t>
+          <t>Stay till the end: FREE 1-on-1 consultation + special announcement</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Quick quiz! Type T or F 👇</t>
+          <t>Quick quiz! Type T or F</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
@@ -770,7 +770,7 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>FALSE ✅</t>
+          <t>FALSE</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -808,7 +808,7 @@
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>FALSE ✅ ₹1 Crore+ in 150 days with a faceless product</t>
+          <t>FALSE. ₹1 Crore+ in 150 days with a faceless product</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>FALSE ✅ Just chat!</t>
+          <t>FALSE. Just chat!</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="C20" s="6" t="inlineStr">
         <is>
-          <t>FALSE ✅ ₹8,435 ads ➡️ ₹12 Lakh revenue</t>
+          <t>FALSE. ₹8,435 ads &gt;&gt; ₹12 Lakh revenue</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
@@ -941,7 +941,7 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>TRUE ✅ AI removes the hard work, not your effort 💪</t>
+          <t>TRUE. AI removes the hard work, not your effort</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>How many did you get right? 🧐</t>
+          <t>How many did you get right?</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Ready for the LIVE demo? Type EXCITED 🔥</t>
+          <t>Ready for the LIVE demo? Type EXCITED</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -998,7 +998,7 @@
       </c>
       <c r="C26" s="6" t="inlineStr">
         <is>
-          <t>Drop your business idea 👇 we'll build it LIVE</t>
+          <t>Drop your business idea in the chat, we'll build it LIVE</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="C28" s="6" t="inlineStr">
         <is>
-          <t>Live on the internet in under 2 minutes ⚡</t>
+          <t>Live on the internet in under 2 minutes</t>
         </is>
       </c>
       <c r="D28" s="8" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Payments live – UPI, Card, EMI, Net Banking. Type WOW 🤯</t>
+          <t>Payments live – UPI, Card, EMI, Net Banking. Type WOW</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
@@ -1074,7 +1074,7 @@
       </c>
       <c r="C30" s="6" t="inlineStr">
         <is>
-          <t>Bump offer = Amazon's "add a screen guard?" 📱 More money from every customer</t>
+          <t>Bump offer works like Amazon's "add a screen guard?" – more money from every customer</t>
         </is>
       </c>
       <c r="D30" s="8" t="inlineStr">
@@ -1131,7 +1131,7 @@
       </c>
       <c r="C33" s="6" t="inlineStr">
         <is>
-          <t>FlexiGenie app on Play Store &amp; App Store 📲 Build your business from your phone</t>
+          <t>FlexiGenie app on Play Store &amp; App Store. Build your business from your phone</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Keep noting down your questions 📝 Sir will answer them at the end. Keep your WhatsApp number ready too 😉</t>
+          <t>Keep noting down your questions. Sir will answer them at the end. Keep your WhatsApp number ready too</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
@@ -1188,7 +1188,7 @@
       </c>
       <c r="C36" s="6" t="inlineStr">
         <is>
-          <t>First Crore at 24 🔥</t>
+          <t>First Crore at 24</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
@@ -1207,7 +1207,7 @@
       </c>
       <c r="C37" s="6" t="inlineStr">
         <is>
-          <t>From selling coupons door-to-door in Dehradun 🙏</t>
+          <t>From selling coupons door-to-door in Dehradun</t>
         </is>
       </c>
       <c r="D37" s="8" t="inlineStr">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="C38" s="6" t="inlineStr">
         <is>
-          <t>Background doesn't matter. Skills do 💯</t>
+          <t>Background doesn't matter. Skills do</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>Model #1 – Faceless Digital Product 📘 ₹1 Crore in 150 days</t>
+          <t>Model #1 – Faceless Digital Product. ₹1 Crore in 150 days</t>
         </is>
       </c>
       <c r="D39" s="8" t="inlineStr">
@@ -1283,7 +1283,7 @@
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>Model #2 – Selling Courses 🎓 Type 1 if you want to sell a course</t>
+          <t>Model #2 – Selling Courses. Type 1 if you want to sell a course</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="C42" s="6" t="inlineStr">
         <is>
-          <t>₹3,000 ad spend ➡️ ₹1.4 Lakh in ONE day</t>
+          <t>₹3,000 ad spend &gt;&gt; ₹1.4 Lakh in ONE day</t>
         </is>
       </c>
       <c r="D42" s="8" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>Model #3 – Consultation 💼 ₹10K ads ➡️ ₹1.5 Lakh</t>
+          <t>Model #3 – Consultation. ₹10K ads &gt;&gt; ₹1.5 Lakh</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
@@ -1340,7 +1340,7 @@
       </c>
       <c r="C44" s="6" t="inlineStr">
         <is>
-          <t>Model #4 – Local Business 🏪 Restaurant, gym, salon, clinic, real estate. Local business owners, type Yes</t>
+          <t>Model #4 – Local Business. Restaurant, gym, salon, clinic, real estate. Local business owners, type Yes</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
@@ -1359,7 +1359,7 @@
       </c>
       <c r="C45" s="6" t="inlineStr">
         <is>
-          <t>Model #5 – Freelancing / Agency 💻 ₹2 Lakh per funnel</t>
+          <t>Model #5 – Freelancing / Agency. ₹2 Lakh per funnel</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
@@ -1378,7 +1378,7 @@
       </c>
       <c r="C46" s="6" t="inlineStr">
         <is>
-          <t>Which model fits YOU? Type 1, 2, 3, 4 or 5 👇</t>
+          <t>Which model fits YOU? Type 1, 2, 3, 4 or 5</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="C47" s="6" t="inlineStr">
         <is>
-          <t>Excited? Type 111 🔥</t>
+          <t>Excited? Type 111</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="C50" s="6" t="inlineStr">
         <is>
-          <t>No guesswork – copy what's already working ✅</t>
+          <t>No guesswork – copy what's already working</t>
         </is>
       </c>
       <c r="D50" s="7" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="C52" s="6" t="inlineStr">
         <is>
-          <t>30 days 100% money-back guarantee ✅ Zero risk</t>
+          <t>30 days 100% money-back guarantee. Zero risk</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="C55" s="6" t="inlineStr">
         <is>
-          <t>24x7 support – reply in 3 minutes + 3 one-on-one calls 📞</t>
+          <t>24x7 support – reply in 3 minutes + 3 one-on-one calls</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>TODAY ONLY – $447 🔥
+          <t>TODAY ONLY – $447
 https://flexifunnels.com/now</t>
         </is>
       </c>
@@ -1645,12 +1645,12 @@
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Confused which model fits YOU? Drop your WhatsApp number 👇 A senior mentor will call and map your personal roadmap – FREE</t>
+          <t>Confused which model fits YOU? Drop your WhatsApp number. A senior mentor will call and map your personal roadmap – FREE</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -1664,12 +1664,12 @@
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>Need EMI? Drop your number – our team will find the easiest EMI plan for you in 2 minutes ✅</t>
+          <t>Need EMI? Drop your number – our team will find the easiest EMI plan for you in 2 minutes</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -1683,7 +1683,7 @@
       </c>
       <c r="C62" s="6" t="inlineStr">
         <is>
-          <t>Rs. 59/day – less than a chai &amp; samosa ☕</t>
+          <t>Rs. 59/day – less than a chai &amp; samosa</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
@@ -1702,7 +1702,7 @@
       </c>
       <c r="C63" s="6" t="inlineStr">
         <is>
-          <t>Bajaj Finance EMI – no credit card needed ✅</t>
+          <t>Bajaj Finance EMI – no credit card needed</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
@@ -1721,12 +1721,12 @@
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>Not ready to pay? Totally fine 🙏 Just drop your number. Clarity is free, the decision is yours</t>
+          <t>Not ready to pay? Totally fine. Just drop your number. Clarity is free, the decision is yours</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -1740,7 +1740,7 @@
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>First 30 only – UNLIMITED funnels &amp; pages + 200 Genie actions/month 🎁</t>
+          <t>First 30 only – UNLIMITED funnels &amp; pages + 200 Genie actions/month</t>
         </is>
       </c>
       <c r="D65" s="12" t="inlineStr">
@@ -1759,12 +1759,12 @@
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>Want a First 30 seat but stuck on payment? Drop your number – our team will help you lock it 🔒</t>
+          <t>Want a First 30 seat but stuck on payment? Drop your number – our team will help you lock it</t>
         </is>
       </c>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -1778,7 +1778,7 @@
       </c>
       <c r="C67" s="6" t="inlineStr">
         <is>
-          <t>Gold ticket worth ₹12,000 FREE 🎟️ + 14 months access</t>
+          <t>Gold ticket worth ₹12,000 FREE + 14 months access</t>
         </is>
       </c>
       <c r="D67" s="12" t="inlineStr">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>8 seats GONE – 22 left ⏳</t>
+          <t>8 seats GONE – 22 left</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
@@ -1816,12 +1816,12 @@
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Don't lose your seat while you're still thinking 😅 Drop your number – our team will call you right now</t>
+          <t>Don't lose your seat while you're still thinking. Drop your number – our team will call you right now</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -1835,7 +1835,7 @@
       </c>
       <c r="C70" s="6" t="inlineStr">
         <is>
-          <t>15 Days First Sale Challenge 🏆</t>
+          <t>15 Days First Sale Challenge</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
@@ -1854,12 +1854,12 @@
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Every success story you saw today started with one small step. Yours can start with a message 👉 drop your number</t>
+          <t>Every success story you saw today started with one small step. Yours can start with a message – drop your number</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -1911,12 +1911,12 @@
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>Need to discuss at home first? 👨‍👩‍👧 Drop your number – our team can explain everything to your family on the call too</t>
+          <t>Need to discuss at home first? Drop your number – our team can explain everything to your family on the call too</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1949,7 @@
       </c>
       <c r="C76" s="6" t="inlineStr">
         <is>
-          <t>Can't pay the full amount? Token ₹2,000–5,000 locks your price &amp; bonuses 👉 https://sb.flexifunnels.com/reserve2k</t>
+          <t>Can't pay the full amount? Token ₹2,000–5,000 locks your price &amp; bonuses: https://sb.flexifunnels.com/reserve2k</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="D77" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -1987,7 +1987,7 @@
       </c>
       <c r="C78" s="6" t="inlineStr">
         <is>
-          <t>300 leads × 2% = ₹1.8 Lakh/day 📈</t>
+          <t>300 leads × 2% = ₹1.8 Lakh/day</t>
         </is>
       </c>
       <c r="D78" s="8" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="D79" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2044,12 +2044,12 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Starting from zero? So did every person you saw today 🙌 Drop your number – we'll start with you from step 1</t>
+          <t>Starting from zero? So did every person you saw today. Drop your number – we'll start with you from step 1</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2063,12 +2063,12 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>No question is too small 🙋 Drop your question + your number – personal answer from our team</t>
+          <t>No question is too small. Drop your question + your number – personal answer from our team</t>
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2120,12 +2120,12 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Wondering how to do this alongside your job? Drop your number – our team will plan your 1 hour/day routine with you ⏰</t>
+          <t>Wondering how to do this alongside your job? Drop your number – our team will plan your 1 hour/day routine with you</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2158,12 +2158,12 @@
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>Stuck on the payment page? Drop your number – we'll stay on the call till it's done ✅</t>
+          <t>Stuck on the payment page? Drop your number – we'll stay on the call till it's done</t>
         </is>
       </c>
       <c r="D87" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>Only 6 seats left ⏳ Take Action Now</t>
+          <t>Only 6 seats left. Take Action Now</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
@@ -2196,12 +2196,12 @@
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>No spam. No pressure. Just one call from a senior mentor. Drop your number 📞</t>
+          <t>No spam. No pressure. Just one call from a senior mentor. Drop your number</t>
         </is>
       </c>
       <c r="D89" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2215,7 +2215,7 @@
       </c>
       <c r="C90" s="6" t="inlineStr">
         <is>
-          <t>What's your first income goal? Type it 🎯</t>
+          <t>What's your first income goal? Type it</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
@@ -2253,12 +2253,12 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>Typed your goal? Now drop your number – a mentor will break it into a step-by-step plan 🎯</t>
+          <t>Typed your goal? Now drop your number – a mentor will break it into a step-by-step plan</t>
         </is>
       </c>
       <c r="D92" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2291,12 +2291,12 @@
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>We already have your number from registration 👆 Typing it here shows you're SERIOUS. Serious people get the first call 📞</t>
+          <t>We already have your number from registration. Typing it here shows you're SERIOUS. Serious people get the first call</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2310,7 +2310,7 @@
       </c>
       <c r="C95" s="6" t="inlineStr">
         <is>
-          <t>AI video with your own face &amp; voice 🤯 Type WOW</t>
+          <t>AI video with your own face &amp; voice. Type WOW</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
@@ -2348,7 +2348,7 @@
       </c>
       <c r="C97" s="6" t="inlineStr">
         <is>
-          <t>Drop your questions now 👇 Sir is answering live</t>
+          <t>Drop your questions now. Sir is answering live</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
@@ -2367,7 +2367,7 @@
       </c>
       <c r="C98" s="6" t="inlineStr">
         <is>
-          <t>Beginner? Works for you ✅ | Job? 60 min/day is enough ✅ | No product? Faceless product in 1 day ✅</t>
+          <t>Beginner? Works for you | Job? 60 min/day is enough | No product? Faceless product in 1 day</t>
         </is>
       </c>
       <c r="D98" s="9" t="inlineStr">
@@ -2386,12 +2386,12 @@
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>Your situation is unique. Drop your number – we'll tell you honestly whether this is right for you 🤝</t>
+          <t>Your situation is unique. Drop your number – we'll tell you honestly whether this is right for you</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2424,7 +2424,7 @@
       </c>
       <c r="C101" s="6" t="inlineStr">
         <is>
-          <t>Domain connect FREE + hosting included 🌐</t>
+          <t>Domain connect FREE + hosting included</t>
         </is>
       </c>
       <c r="D101" s="9" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="C102" s="6" t="inlineStr">
         <is>
-          <t>Next 5 minutes only – complete UNLIMITED access 🔓</t>
+          <t>Next 5 minutes only – complete UNLIMITED access</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
@@ -2462,12 +2462,12 @@
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>No business idea yet? Drop your number – a mentor will help you find one that fits your skills 💡</t>
+          <t>No business idea yet? Drop your number – a mentor will help you find one that fits your skills</t>
         </is>
       </c>
       <c r="D103" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2481,12 +2481,12 @@
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
-          <t>Clinic, coaching, salon, factory, shop… drop your number + your business type – we'll show you how it goes online 🚀</t>
+          <t>Clinic, coaching, salon, factory, shop… drop your number + your business type – we'll show you how it goes online</t>
         </is>
       </c>
       <c r="D104" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2500,7 +2500,7 @@
       </c>
       <c r="C105" s="6" t="inlineStr">
         <is>
-          <t>What do you have to lose? 30 days money-back guarantee ✅</t>
+          <t>What do you have to lose? 30 days money-back guarantee</t>
         </is>
       </c>
       <c r="D105" s="9" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="C106" s="6" t="inlineStr">
         <is>
-          <t>1% transaction fee – we win only when you win 🤝</t>
+          <t>1% transaction fee – we win only when you win</t>
         </is>
       </c>
       <c r="D106" s="9" t="inlineStr">
@@ -2557,12 +2557,12 @@
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>Typed 1? That's your first step. Step 2: drop your number 👇</t>
+          <t>Typed 1? That's your first step. Step 2: drop your number</t>
         </is>
       </c>
       <c r="D108" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2595,7 +2595,7 @@
       </c>
       <c r="C110" s="6" t="inlineStr">
         <is>
-          <t>Deal? Type Yes 🤝</t>
+          <t>Deal? Type Yes</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
@@ -2614,12 +2614,12 @@
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>Is it a deal? 🤝 Seal it – drop your number</t>
+          <t>Is it a deal? Seal it – drop your number</t>
         </is>
       </c>
       <c r="D111" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2633,7 +2633,7 @@
       </c>
       <c r="C112" s="6" t="inlineStr">
         <is>
-          <t>Closing soon – bonuses end with the session ⏳</t>
+          <t>Closing soon – bonuses end with the session</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
@@ -2652,12 +2652,12 @@
       </c>
       <c r="C113" s="11" t="inlineStr">
         <is>
-          <t>Session ends in 5 minutes. Bonuses end with it. Drop your number to still get help ⏳</t>
+          <t>Session ends in 5 minutes. Bonuses end with it. Drop your number to still get help</t>
         </is>
       </c>
       <c r="D113" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2733,7 +2733,7 @@
       </c>
       <c r="D117" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2747,7 +2747,7 @@
       </c>
       <c r="C118" s="6" t="inlineStr">
         <is>
-          <t>98% never take action. Be the 2% 💪</t>
+          <t>98% never take action. Be the 2%</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
@@ -2766,12 +2766,12 @@
       </c>
       <c r="C119" s="11" t="inlineStr">
         <is>
-          <t>Same situation one year from now, or one call today? Drop your number 📞</t>
+          <t>Same situation one year from now, or one call today? Drop your number</t>
         </is>
       </c>
       <c r="D119" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2809,7 +2809,7 @@
       </c>
       <c r="D121" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2823,7 @@
       </c>
       <c r="C122" s="6" t="inlineStr">
         <is>
-          <t>What if I fly? 🦅</t>
+          <t>What if I fly?</t>
         </is>
       </c>
       <c r="D122" s="7" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="C123" s="6" t="inlineStr">
         <is>
-          <t>LAST CALL 📢</t>
+          <t>LAST CALL</t>
         </is>
       </c>
       <c r="D123" s="12" t="inlineStr">
@@ -2861,12 +2861,12 @@
       </c>
       <c r="C124" s="11" t="inlineStr">
         <is>
-          <t>Last call. If you don't drop your number today, you'll still be thinking about it tomorrow. Drop it now 👇</t>
+          <t>Last call. If you don't drop your number today, you'll still be thinking about it tomorrow. Drop it now</t>
         </is>
       </c>
       <c r="D124" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2899,12 +2899,12 @@
       </c>
       <c r="C126" s="11" t="inlineStr">
         <is>
-          <t>Your decision, your life – not anyone else's. Drop your number &amp; decide with full clarity 💯</t>
+          <t>Your decision, your life – not anyone else's. Drop your number &amp; decide with full clarity</t>
         </is>
       </c>
       <c r="D126" s="11" t="inlineStr">
         <is>
-          <t>📞 NUMBER DROP</t>
+          <t>NUMBER DROP</t>
         </is>
       </c>
     </row>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="C128" s="6" t="inlineStr">
         <is>
-          <t>Stay till the end – something special coming 🎁</t>
+          <t>Stay till the end – something special coming</t>
         </is>
       </c>
       <c r="D128" s="7" t="inlineStr">
@@ -3092,7 +3092,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Confused which model fits YOU? Drop your WhatsApp number 👇 A senior mentor will call and map your personal roadmap – FREE</t>
+          <t>Confused which model fits YOU? Drop your WhatsApp number. A senior mentor will call and map your personal roadmap – FREE</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Not ready to pay? Totally fine 🙏 Just drop your number. Clarity is free, the decision is yours</t>
+          <t>Not ready to pay? Totally fine. Just drop your number. Clarity is free, the decision is yours</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -3126,7 +3126,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Your situation is unique. Drop your number – we'll tell you honestly whether this is right for you 🤝</t>
+          <t>Your situation is unique. Drop your number – we'll tell you honestly whether this is right for you</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Need EMI? Drop your number – our team will find the easiest EMI plan for you in 2 minutes ✅</t>
+          <t>Need EMI? Drop your number – our team will find the easiest EMI plan for you in 2 minutes</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Stuck on the payment page? Drop your number – we'll stay on the call till it's done ✅</t>
+          <t>Stuck on the payment page? Drop your number – we'll stay on the call till it's done</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Need to discuss at home first? 👨‍👩‍👧 Drop your number – our team can explain everything to your family on the call too</t>
+          <t>Need to discuss at home first? Drop your number – our team can explain everything to your family on the call too</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Wondering how to do this alongside your job? Drop your number – our team will plan your 1 hour/day routine with you ⏰</t>
+          <t>Wondering how to do this alongside your job? Drop your number – our team will plan your 1 hour/day routine with you</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -3245,7 +3245,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Starting from zero? So did every person you saw today 🙌 Drop your number – we'll start with you from step 1</t>
+          <t>Starting from zero? So did every person you saw today. Drop your number – we'll start with you from step 1</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -3262,7 +3262,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>No question is too small 🙋 Drop your question + your number – personal answer from our team</t>
+          <t>No question is too small. Drop your question + your number – personal answer from our team</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>No business idea yet? Drop your number – a mentor will help you find one that fits your skills 💡</t>
+          <t>No business idea yet? Drop your number – a mentor will help you find one that fits your skills</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Clinic, coaching, salon, factory, shop… drop your number + your business type – we'll show you how it goes online 🚀</t>
+          <t>Clinic, coaching, salon, factory, shop… drop your number + your business type – we'll show you how it goes online</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Typed your goal? Now drop your number – a mentor will break it into a step-by-step plan 🎯</t>
+          <t>Typed your goal? Now drop your number – a mentor will break it into a step-by-step plan</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Typed 1? That's your first step. Step 2: drop your number 👇</t>
+          <t>Typed 1? That's your first step. Step 2: drop your number</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Is it a deal? 🤝 Seal it – drop your number</t>
+          <t>Is it a deal? Seal it – drop your number</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>We already have your number from registration 👆 Typing it here shows you're SERIOUS. Serious people get the first call 📞</t>
+          <t>We already have your number from registration. Typing it here shows you're SERIOUS. Serious people get the first call</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -3415,7 +3415,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Every success story you saw today started with one small step. Yours can start with a message 👉 drop your number</t>
+          <t>Every success story you saw today started with one small step. Yours can start with a message – drop your number</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -3432,7 +3432,7 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>No spam. No pressure. Just one call from a senior mentor. Drop your number 📞</t>
+          <t>No spam. No pressure. Just one call from a senior mentor. Drop your number</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -3449,7 +3449,7 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Don't lose your seat while you're still thinking 😅 Drop your number – our team will call you right now</t>
+          <t>Don't lose your seat while you're still thinking. Drop your number – our team will call you right now</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -3466,7 +3466,7 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Want a First 30 seat but stuck on payment? Drop your number – our team will help you lock it 🔒</t>
+          <t>Want a First 30 seat but stuck on payment? Drop your number – our team will help you lock it</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Session ends in 5 minutes. Bonuses end with it. Drop your number to still get help ⏳</t>
+          <t>Session ends in 5 minutes. Bonuses end with it. Drop your number to still get help</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -3500,7 +3500,7 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Same situation one year from now, or one call today? Drop your number 📞</t>
+          <t>Same situation one year from now, or one call today? Drop your number</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Last call. If you don't drop your number today, you'll still be thinking about it tomorrow. Drop it now 👇</t>
+          <t>Last call. If you don't drop your number today, you'll still be thinking about it tomorrow. Drop it now</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -3534,7 +3534,7 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Your decision, your life – not anyone else's. Drop your number &amp; decide with full clarity 💯</t>
+          <t>Your decision, your life – not anyone else's. Drop your number &amp; decide with full clarity</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Thank you {Name}, {Name} &amp; {Name} 🙏 Our team is calling you shortly. Others, drop your number 👇</t>
+          <t>Thank you {Name}, {Name} &amp; {Name}. Our team is calling you shortly. Others, drop your number</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -3745,7 +3745,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Yes, {Name}, you're in the First 30 🎉</t>
+          <t>Yes, {Name}, you're in the First 30</t>
         </is>
       </c>
     </row>
@@ -3986,7 +3986,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>No coding, no tech – you just chat with FlexiGenie and it builds everything 💬</t>
+          <t>No coding, no tech – you just chat with FlexiGenie and it builds everything</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Start with a faceless digital product – create it in a single day with our custom GPTs 📘</t>
+          <t>Start with a faceless digital product – create it in a single day with our custom GPTs</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>60 minutes a day is more than enough. Many members started while working full-time ⏰</t>
+          <t>60 minutes a day is more than enough. Many members started while working full-time</t>
         </is>
       </c>
     </row>
@@ -4022,7 +4022,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>EMI from Rs. 59/day or token payment available. Share your contact number 🙏</t>
+          <t>EMI from Rs. 59/day or token payment available. Share your contact number</t>
         </is>
       </c>
     </row>
@@ -4034,7 +4034,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Bajaj Finance EMI available – no credit card needed ✅</t>
+          <t>Bajaj Finance EMI available – no credit card needed</t>
         </is>
       </c>
     </row>
@@ -4046,7 +4046,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>30 days ironclad 100% money-back guarantee – no questions asked ✅</t>
+          <t>30 days ironclad 100% money-back guarantee – no questions asked</t>
         </is>
       </c>
     </row>
@@ -4058,7 +4058,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Everybody starts from ZERO – 4,700+ success stories started exactly where you are 💪</t>
+          <t>Everybody starts from ZERO – 4,700+ success stories started exactly where you are</t>
         </is>
       </c>
     </row>
@@ -4094,7 +4094,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>We earn 1% on transactions – we win only when you win 🤝</t>
+          <t>We earn 1% on transactions – we win only when you win</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Yes – connect your own domain FREE, hosting included 🌐</t>
+          <t>Yes – connect your own domain FREE, hosting included</t>
         </is>
       </c>
     </row>
@@ -4118,7 +4118,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>You don't need to learn AI or computers – just chat like WhatsApp 📱</t>
+          <t>You don't need to learn AI or computers – just chat like WhatsApp</t>
         </is>
       </c>
     </row>
@@ -4130,7 +4130,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>24x7 live chat – real humans, reply within 3 minutes + 3 one-on-one calls 📞</t>
+          <t>24x7 live chat – real humans, reply within 3 minutes + 3 one-on-one calls</t>
         </is>
       </c>
     </row>
@@ -4142,7 +4142,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Yes – sub-user access with controlled permissions 👥</t>
+          <t>Yes – sub-user access with controlled permissions</t>
         </is>
       </c>
     </row>
@@ -4154,7 +4154,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>You don't need to be the best – just one step ahead of the people you help 🙌</t>
+          <t>You don't need to be the best – just one step ahead of the people you help</t>
         </is>
       </c>
     </row>
@@ -4166,7 +4166,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Possible from day one – 15 Days First Sale Challenge helps you crack it 🏆</t>
+          <t>Possible from day one – 15 Days First Sale Challenge helps you crack it</t>
         </is>
       </c>
     </row>
@@ -4178,7 +4178,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>$447 is today only – $697 tomorrow, $997 day after ⏳</t>
+          <t>$447 is today only – $697 tomorrow, $997 day after</t>
         </is>
       </c>
     </row>
@@ -4190,7 +4190,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Yes – live chat support + live weekly Q&amp;A sessions 🎥</t>
+          <t>Yes – live chat support + live weekly Q&amp;A sessions</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add minimal emojis to urgency and number-drop chat lines
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013vbY3qGkzmvkM4RiAXuEBt
</commit_message>
<xml_diff>
--- a/FlexiGenie_Webinar_Chat_Sheet.xlsx
+++ b/FlexiGenie_Webinar_Chat_Sheet.xlsx
@@ -1606,7 +1606,7 @@
       </c>
       <c r="C58" s="6" t="inlineStr">
         <is>
-          <t>TODAY ONLY – $447
+          <t>TODAY ONLY – $447 🔥
 https://flexifunnels.com/now</t>
         </is>
       </c>
@@ -1645,7 +1645,7 @@
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Confused which model fits YOU? Drop your WhatsApp number. A senior mentor will call and map your personal roadmap – FREE</t>
+          <t>Confused which model fits YOU? Drop your WhatsApp number. A senior mentor will call and map your personal roadmap – FREE 👇</t>
         </is>
       </c>
       <c r="D60" s="11" t="inlineStr">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>Need EMI? Drop your number – our team will find the easiest EMI plan for you in 2 minutes</t>
+          <t>Need EMI? Drop your number – our team will find the easiest EMI plan for you in 2 minutes 📞</t>
         </is>
       </c>
       <c r="D61" s="11" t="inlineStr">
@@ -1721,7 +1721,7 @@
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>Not ready to pay? Totally fine. Just drop your number. Clarity is free, the decision is yours</t>
+          <t>Not ready to pay? Totally fine. Just drop your number. Clarity is free, the decision is yours 🙏</t>
         </is>
       </c>
       <c r="D64" s="11" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="C65" s="6" t="inlineStr">
         <is>
-          <t>First 30 only – UNLIMITED funnels &amp; pages + 200 Genie actions/month</t>
+          <t>First 30 only – UNLIMITED funnels &amp; pages + 200 Genie actions/month 🎁</t>
         </is>
       </c>
       <c r="D65" s="12" t="inlineStr">
@@ -1759,7 +1759,7 @@
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>Want a First 30 seat but stuck on payment? Drop your number – our team will help you lock it</t>
+          <t>Want a First 30 seat but stuck on payment? Drop your number – our team will help you lock it 🔒</t>
         </is>
       </c>
       <c r="D66" s="11" t="inlineStr">
@@ -1797,7 +1797,7 @@
       </c>
       <c r="C68" s="6" t="inlineStr">
         <is>
-          <t>8 seats GONE – 22 left</t>
+          <t>8 seats GONE – 22 left ⏳</t>
         </is>
       </c>
       <c r="D68" s="12" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Don't lose your seat while you're still thinking. Drop your number – our team will call you right now</t>
+          <t>Don't lose your seat while you're still thinking. Drop your number – our team will call you right now ⏳</t>
         </is>
       </c>
       <c r="D69" s="11" t="inlineStr">
@@ -1854,7 +1854,7 @@
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Every success story you saw today started with one small step. Yours can start with a message – drop your number</t>
+          <t>Every success story you saw today started with one small step. Yours can start with a message – drop your number 👇</t>
         </is>
       </c>
       <c r="D71" s="11" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="C73" s="6" t="inlineStr">
         <is>
-          <t>17 seats left in First 30</t>
+          <t>17 seats left in First 30 ⏳</t>
         </is>
       </c>
       <c r="D73" s="12" t="inlineStr">
@@ -1911,7 +1911,7 @@
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>Need to discuss at home first? Drop your number – our team can explain everything to your family on the call too</t>
+          <t>Need to discuss at home first? Drop your number – our team can explain everything to your family on the call too 📞</t>
         </is>
       </c>
       <c r="D74" s="11" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Type 1 + drop your number – our team will help you with the token &amp; balance payment</t>
+          <t>Type 1 + drop your number – our team will help you with the token &amp; balance payment 👇</t>
         </is>
       </c>
       <c r="D77" s="11" t="inlineStr">
@@ -2006,7 +2006,7 @@
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>How much should YOU spend on ads? Drop your number – a mentor will work it out for YOUR business</t>
+          <t>How much should YOU spend on ads? Drop your number – a mentor will work it out for YOUR business 👇</t>
         </is>
       </c>
       <c r="D79" s="11" t="inlineStr">
@@ -2025,7 +2025,7 @@
       </c>
       <c r="C80" s="6" t="inlineStr">
         <is>
-          <t>12 seats left</t>
+          <t>12 seats left ⏳</t>
         </is>
       </c>
       <c r="D80" s="12" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Starting from zero? So did every person you saw today. Drop your number – we'll start with you from step 1</t>
+          <t>Starting from zero? So did every person you saw today. Drop your number – we'll start with you from step 1 🙌</t>
         </is>
       </c>
       <c r="D81" s="11" t="inlineStr">
@@ -2063,7 +2063,7 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>No question is too small. Drop your question + your number – personal answer from our team</t>
+          <t>No question is too small. Drop your question + your number – personal answer from our team 👇</t>
         </is>
       </c>
       <c r="D82" s="11" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="C84" s="6" t="inlineStr">
         <is>
-          <t>9 seats left</t>
+          <t>9 seats left ⏳</t>
         </is>
       </c>
       <c r="D84" s="12" t="inlineStr">
@@ -2120,7 +2120,7 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Wondering how to do this alongside your job? Drop your number – our team will plan your 1 hour/day routine with you</t>
+          <t>Wondering how to do this alongside your job? Drop your number – our team will plan your 1 hour/day routine with you 📞</t>
         </is>
       </c>
       <c r="D85" s="11" t="inlineStr">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>Stuck on the payment page? Drop your number – we'll stay on the call till it's done</t>
+          <t>Stuck on the payment page? Drop your number – we'll stay on the call till it's done 📞</t>
         </is>
       </c>
       <c r="D87" s="11" t="inlineStr">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="C88" s="6" t="inlineStr">
         <is>
-          <t>Only 6 seats left. Take Action Now</t>
+          <t>Only 6 seats left. Take Action Now ⏳</t>
         </is>
       </c>
       <c r="D88" s="12" t="inlineStr">
@@ -2196,7 +2196,7 @@
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>No spam. No pressure. Just one call from a senior mentor. Drop your number</t>
+          <t>No spam. No pressure. Just one call from a senior mentor. Drop your number 📞</t>
         </is>
       </c>
       <c r="D89" s="11" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>Typed your goal? Now drop your number – a mentor will break it into a step-by-step plan</t>
+          <t>Typed your goal? Now drop your number – a mentor will break it into a step-by-step plan 🎯</t>
         </is>
       </c>
       <c r="D92" s="11" t="inlineStr">
@@ -2272,7 +2272,7 @@
       </c>
       <c r="C93" s="6" t="inlineStr">
         <is>
-          <t>Only 2 seats left!</t>
+          <t>Only 2 seats left! 🚨</t>
         </is>
       </c>
       <c r="D93" s="12" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>We already have your number from registration. Typing it here shows you're SERIOUS. Serious people get the first call</t>
+          <t>We already have your number from registration. Typing it here shows you're SERIOUS. Serious people get the first call 📞</t>
         </is>
       </c>
       <c r="D94" s="11" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="C96" s="6" t="inlineStr">
         <is>
-          <t>LAST 2 SEATS</t>
+          <t>LAST 2 SEATS 🚨</t>
         </is>
       </c>
       <c r="D96" s="12" t="inlineStr">
@@ -2386,7 +2386,7 @@
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>Your situation is unique. Drop your number – we'll tell you honestly whether this is right for you</t>
+          <t>Your situation is unique. Drop your number – we'll tell you honestly whether this is right for you 🤝</t>
         </is>
       </c>
       <c r="D99" s="11" t="inlineStr">
@@ -2405,7 +2405,7 @@
       </c>
       <c r="C100" s="6" t="inlineStr">
         <is>
-          <t>LAST SEAT in First 30! Type 1</t>
+          <t>LAST SEAT in First 30! Type 1 🚨</t>
         </is>
       </c>
       <c r="D100" s="12" t="inlineStr">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="C102" s="6" t="inlineStr">
         <is>
-          <t>Next 5 minutes only – complete UNLIMITED access</t>
+          <t>Next 5 minutes only – complete UNLIMITED access ⏰</t>
         </is>
       </c>
       <c r="D102" s="12" t="inlineStr">
@@ -2462,7 +2462,7 @@
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>No business idea yet? Drop your number – a mentor will help you find one that fits your skills</t>
+          <t>No business idea yet? Drop your number – a mentor will help you find one that fits your skills 👇</t>
         </is>
       </c>
       <c r="D103" s="11" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
-          <t>Clinic, coaching, salon, factory, shop… drop your number + your business type – we'll show you how it goes online</t>
+          <t>Clinic, coaching, salon, factory, shop… drop your number + your business type – we'll show you how it goes online 👇</t>
         </is>
       </c>
       <c r="D104" s="11" t="inlineStr">
@@ -2557,7 +2557,7 @@
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>Typed 1? That's your first step. Step 2: drop your number</t>
+          <t>Typed 1? That's your first step. Step 2: drop your number 👇</t>
         </is>
       </c>
       <c r="D108" s="11" t="inlineStr">
@@ -2614,7 +2614,7 @@
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>Is it a deal? Seal it – drop your number</t>
+          <t>Is it a deal? Seal it – drop your number 🤝</t>
         </is>
       </c>
       <c r="D111" s="11" t="inlineStr">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="C112" s="6" t="inlineStr">
         <is>
-          <t>Closing soon – bonuses end with the session</t>
+          <t>Closing soon – bonuses end with the session ⏰</t>
         </is>
       </c>
       <c r="D112" s="12" t="inlineStr">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="C113" s="11" t="inlineStr">
         <is>
-          <t>Session ends in 5 minutes. Bonuses end with it. Drop your number to still get help</t>
+          <t>Session ends in 5 minutes. Bonuses end with it. Drop your number to still get help ⏳</t>
         </is>
       </c>
       <c r="D113" s="11" t="inlineStr">
@@ -2728,7 +2728,7 @@
       </c>
       <c r="C117" s="11" t="inlineStr">
         <is>
-          <t>Something keeping you stuck? Type 1 &amp; drop your number – let's remove it together</t>
+          <t>Something keeping you stuck? Type 1 &amp; drop your number – let's remove it together 👇</t>
         </is>
       </c>
       <c r="D117" s="11" t="inlineStr">
@@ -2766,7 +2766,7 @@
       </c>
       <c r="C119" s="11" t="inlineStr">
         <is>
-          <t>Same situation one year from now, or one call today? Drop your number</t>
+          <t>Same situation one year from now, or one call today? Drop your number 📞</t>
         </is>
       </c>
       <c r="D119" s="11" t="inlineStr">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="C121" s="11" t="inlineStr">
         <is>
-          <t>Bajaj Finance EMI – done in 30 minutes. Drop your number</t>
+          <t>Bajaj Finance EMI – done in 30 minutes. Drop your number 📞</t>
         </is>
       </c>
       <c r="D121" s="11" t="inlineStr">
@@ -2842,7 +2842,7 @@
       </c>
       <c r="C123" s="6" t="inlineStr">
         <is>
-          <t>LAST CALL</t>
+          <t>LAST CALL 📢</t>
         </is>
       </c>
       <c r="D123" s="12" t="inlineStr">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="C124" s="11" t="inlineStr">
         <is>
-          <t>Last call. If you don't drop your number today, you'll still be thinking about it tomorrow. Drop it now</t>
+          <t>Last call. If you don't drop your number today, you'll still be thinking about it tomorrow. Drop it now 👇</t>
         </is>
       </c>
       <c r="D124" s="11" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="C126" s="11" t="inlineStr">
         <is>
-          <t>Your decision, your life – not anyone else's. Drop your number &amp; decide with full clarity</t>
+          <t>Your decision, your life – not anyone else's. Drop your number &amp; decide with full clarity 👇</t>
         </is>
       </c>
       <c r="D126" s="11" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="C130" s="6" t="inlineStr">
         <is>
-          <t>2 minutes only – https://flexifunnels.com/now</t>
+          <t>2 minutes only – https://flexifunnels.com/now ⏰</t>
         </is>
       </c>
       <c r="D130" s="12" t="inlineStr">
@@ -3092,7 +3092,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>Confused which model fits YOU? Drop your WhatsApp number. A senior mentor will call and map your personal roadmap – FREE</t>
+          <t>Confused which model fits YOU? Drop your WhatsApp number. A senior mentor will call and map your personal roadmap – FREE 👇</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -3109,7 +3109,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Not ready to pay? Totally fine. Just drop your number. Clarity is free, the decision is yours</t>
+          <t>Not ready to pay? Totally fine. Just drop your number. Clarity is free, the decision is yours 🙏</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -3126,7 +3126,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Your situation is unique. Drop your number – we'll tell you honestly whether this is right for you</t>
+          <t>Your situation is unique. Drop your number – we'll tell you honestly whether this is right for you 🤝</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -3143,7 +3143,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Need EMI? Drop your number – our team will find the easiest EMI plan for you in 2 minutes</t>
+          <t>Need EMI? Drop your number – our team will find the easiest EMI plan for you in 2 minutes 📞</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -3160,7 +3160,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Stuck on the payment page? Drop your number – we'll stay on the call till it's done</t>
+          <t>Stuck on the payment page? Drop your number – we'll stay on the call till it's done 📞</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -3177,7 +3177,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Bajaj Finance EMI – done in 30 minutes. Drop your number</t>
+          <t>Bajaj Finance EMI – done in 30 minutes. Drop your number 📞</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Type 1 + drop your number – our team will help you with the token &amp; balance payment</t>
+          <t>Type 1 + drop your number – our team will help you with the token &amp; balance payment 👇</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Need to discuss at home first? Drop your number – our team can explain everything to your family on the call too</t>
+          <t>Need to discuss at home first? Drop your number – our team can explain everything to your family on the call too 📞</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Wondering how to do this alongside your job? Drop your number – our team will plan your 1 hour/day routine with you</t>
+          <t>Wondering how to do this alongside your job? Drop your number – our team will plan your 1 hour/day routine with you 📞</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -3245,7 +3245,7 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Starting from zero? So did every person you saw today. Drop your number – we'll start with you from step 1</t>
+          <t>Starting from zero? So did every person you saw today. Drop your number – we'll start with you from step 1 🙌</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -3262,7 +3262,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>No question is too small. Drop your question + your number – personal answer from our team</t>
+          <t>No question is too small. Drop your question + your number – personal answer from our team 👇</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>No business idea yet? Drop your number – a mentor will help you find one that fits your skills</t>
+          <t>No business idea yet? Drop your number – a mentor will help you find one that fits your skills 👇</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -3296,7 +3296,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>Clinic, coaching, salon, factory, shop… drop your number + your business type – we'll show you how it goes online</t>
+          <t>Clinic, coaching, salon, factory, shop… drop your number + your business type – we'll show you how it goes online 👇</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -3313,7 +3313,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Typed your goal? Now drop your number – a mentor will break it into a step-by-step plan</t>
+          <t>Typed your goal? Now drop your number – a mentor will break it into a step-by-step plan 🎯</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -3330,7 +3330,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>How much should YOU spend on ads? Drop your number – a mentor will work it out for YOUR business</t>
+          <t>How much should YOU spend on ads? Drop your number – a mentor will work it out for YOUR business 👇</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Typed 1? That's your first step. Step 2: drop your number</t>
+          <t>Typed 1? That's your first step. Step 2: drop your number 👇</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
@@ -3364,7 +3364,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>Is it a deal? Seal it – drop your number</t>
+          <t>Is it a deal? Seal it – drop your number 🤝</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
@@ -3381,7 +3381,7 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>Something keeping you stuck? Type 1 &amp; drop your number – let's remove it together</t>
+          <t>Something keeping you stuck? Type 1 &amp; drop your number – let's remove it together 👇</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>We already have your number from registration. Typing it here shows you're SERIOUS. Serious people get the first call</t>
+          <t>We already have your number from registration. Typing it here shows you're SERIOUS. Serious people get the first call 📞</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -3415,7 +3415,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>Every success story you saw today started with one small step. Yours can start with a message – drop your number</t>
+          <t>Every success story you saw today started with one small step. Yours can start with a message – drop your number 👇</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
@@ -3432,7 +3432,7 @@
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>No spam. No pressure. Just one call from a senior mentor. Drop your number</t>
+          <t>No spam. No pressure. Just one call from a senior mentor. Drop your number 📞</t>
         </is>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -3449,7 +3449,7 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Don't lose your seat while you're still thinking. Drop your number – our team will call you right now</t>
+          <t>Don't lose your seat while you're still thinking. Drop your number – our team will call you right now ⏳</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
@@ -3466,7 +3466,7 @@
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>Want a First 30 seat but stuck on payment? Drop your number – our team will help you lock it</t>
+          <t>Want a First 30 seat but stuck on payment? Drop your number – our team will help you lock it 🔒</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr">
@@ -3483,7 +3483,7 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Session ends in 5 minutes. Bonuses end with it. Drop your number to still get help</t>
+          <t>Session ends in 5 minutes. Bonuses end with it. Drop your number to still get help ⏳</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
@@ -3500,7 +3500,7 @@
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>Same situation one year from now, or one call today? Drop your number</t>
+          <t>Same situation one year from now, or one call today? Drop your number 📞</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -3517,7 +3517,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>Last call. If you don't drop your number today, you'll still be thinking about it tomorrow. Drop it now</t>
+          <t>Last call. If you don't drop your number today, you'll still be thinking about it tomorrow. Drop it now 👇</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -3534,7 +3534,7 @@
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>Your decision, your life – not anyone else's. Drop your number &amp; decide with full clarity</t>
+          <t>Your decision, your life – not anyone else's. Drop your number &amp; decide with full clarity 👇</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>Thank you {Name}, {Name} &amp; {Name}. Our team is calling you shortly. Others, drop your number</t>
+          <t>Thank you {Name}, {Name} &amp; {Name}. Our team is calling you shortly. Others, drop your number 🙏</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Update enrolment link in chat sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013vbY3qGkzmvkM4RiAXuEBt
</commit_message>
<xml_diff>
--- a/FlexiGenie_Webinar_Chat_Sheet.xlsx
+++ b/FlexiGenie_Webinar_Chat_Sheet.xlsx
@@ -1607,7 +1607,7 @@
       <c r="C58" s="6" t="inlineStr">
         <is>
           <t>TODAY ONLY – $447 🔥
-https://flexifunnels.com/now</t>
+https://sb.flexifunnels.com/get?id=19029</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
@@ -1873,7 +1873,7 @@
       </c>
       <c r="C72" s="6" t="inlineStr">
         <is>
-          <t>Enrol here: https://flexifunnels.com/now</t>
+          <t>Enrol here: https://sb.flexifunnels.com/get?id=19029</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
@@ -2139,7 +2139,7 @@
       </c>
       <c r="C86" s="6" t="inlineStr">
         <is>
-          <t>EMI Link – https://flexifunnels.com/now (EMIs available on the same link)</t>
+          <t>EMI Link – https://sb.flexifunnels.com/get?id=19029 (EMIs available on the same link)</t>
         </is>
       </c>
       <c r="D86" s="9" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="C116" s="6" t="inlineStr">
         <is>
-          <t>Take Action Now: https://flexifunnels.com/now</t>
+          <t>Take Action Now: https://sb.flexifunnels.com/get?id=19029</t>
         </is>
       </c>
       <c r="D116" s="9" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="C125" s="6" t="inlineStr">
         <is>
-          <t>Rs. 36,999 incl. GST | Rs. 59/day on EMI – https://flexifunnels.com/now</t>
+          <t>Rs. 36,999 incl. GST | Rs. 59/day on EMI – https://sb.flexifunnels.com/get?id=19029</t>
         </is>
       </c>
       <c r="D125" s="9" t="inlineStr">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="C130" s="6" t="inlineStr">
         <is>
-          <t>2 minutes only – https://flexifunnels.com/now ⏰</t>
+          <t>2 minutes only – https://sb.flexifunnels.com/get?id=19029 ⏰</t>
         </is>
       </c>
       <c r="D130" s="12" t="inlineStr">
@@ -3032,7 +3032,7 @@
       </c>
       <c r="C133" s="6" t="inlineStr">
         <is>
-          <t>Final Chance: https://flexifunnels.com/now</t>
+          <t>Final Chance: https://sb.flexifunnels.com/get?id=19029</t>
         </is>
       </c>
       <c r="D133" s="9" t="inlineStr">
@@ -3697,7 +3697,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>{Name}, it's just $447 (Rs. 36,999 incl. GST) today – here's the link: https://flexifunnels.com/now. Kindly share your contact number and our team will guide you.</t>
+          <t>{Name}, it's just $447 (Rs. 36,999 incl. GST) today – here's the link: https://sb.flexifunnels.com/get?id=19029. Kindly share your contact number and our team will guide you.</t>
         </is>
       </c>
     </row>

</xml_diff>